<commit_message>
Fase 4: cierre de resultados del dia
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -941,6 +941,25 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>